<commit_message>
Added Warning and Timeouts
</commit_message>
<xml_diff>
--- a/LoginCPARS/Login-CPARS/Input/Ford Receiving - Input.xlsx
+++ b/LoginCPARS/Login-CPARS/Input/Ford Receiving - Input.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skrishnan1\Videos\Proj\LoginCPARS\Login-CPARS\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4CF8E47-099B-45DE-B282-4322190D0926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700514FE-4C55-446D-92F1-269CC5AC2937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{79995E57-A43A-43D8-997D-622DCF610173}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
     <t>Customer PO</t>
   </si>
@@ -87,6 +87,21 @@
   </si>
   <si>
     <t>RL26442649</t>
+  </si>
+  <si>
+    <t>B45RL26720042</t>
+  </si>
+  <si>
+    <t>2488920</t>
+  </si>
+  <si>
+    <t>060ZA2404</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>RL26720042</t>
   </si>
 </sst>
 </file>
@@ -458,7 +473,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2B01D7E-9741-4D75-B0F4-F372D4AABE30}">
-  <dimension ref="A1:F3"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
@@ -526,6 +542,26 @@
         <v>15</v>
       </c>
     </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>